<commit_message>
Removes code that would exogenously set electrification levels based on input data; updates industry logit coefficient and shareweights
</commit_message>
<xml_diff>
--- a/InputData/indst/IELC/Industrial Eqpt Logit Coefficient.xlsx
+++ b/InputData/indst/IELC/Industrial Eqpt Logit Coefficient.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\indst\IELC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanO'Brien\Models\EPS\US\eps-us\InputData\indst\IELC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4858BA3-C700-4D9F-9521-47DC80F461CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B0B3419-DCCE-447C-B1B0-2B7A92DEEDE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{910269CE-FD31-46D7-B2D8-8AF36ED85333}"/>
+    <workbookView xWindow="-28410" yWindow="390" windowWidth="27510" windowHeight="16560" activeTab="1" xr2:uid="{910269CE-FD31-46D7-B2D8-8AF36ED85333}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -501,14 +501,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E490AE5-9E06-4EDB-8D15-DE332404A026}">
   <dimension ref="A1:B22"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -516,78 +516,78 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>14</v>
       </c>
       <c r="B16" s="5"/>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>20</v>
       </c>
@@ -604,13 +604,13 @@
     <tabColor theme="3" tint="0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.453125" customWidth="1"/>
-    <col min="2" max="2" width="16.1796875" customWidth="1"/>
+    <col min="1" max="1" width="20.42578125" customWidth="1"/>
+    <col min="2" max="2" width="16.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>4</v>
       </c>
@@ -618,12 +618,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
       <c r="B2">
-        <v>-3</v>
+        <v>-6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>